<commit_message>
adding pop in TAZ 7223
</commit_message>
<xml_diff>
--- a/inputs_outputs.xlsx
+++ b/inputs_outputs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\advas\Documents\create_forecast_ad_hoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4978D3F5-92DE-426A-9135-4057F4BDEF74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AE63838-0879-463D-88E2-E5311E5D943D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1160" yWindow="600" windowWidth="21600" windowHeight="12260" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -65,10 +65,10 @@
     <t>base_year</t>
   </si>
   <si>
-    <t>W:\Projects\בהת\גבעת רם - לניסוי בלבד\קבצי עבודה\תחזיות_דמוגרפיות</t>
-  </si>
-  <si>
-    <t>givaat_ram</t>
+    <t>yosh_real_2050</t>
+  </si>
+  <si>
+    <t>W:\Projects\תכניות מרחביות\תוכנית אב יוש_286\קבצי עבודה\תחזיות_דמוגרפיות</t>
   </si>
 </sst>
 </file>
@@ -473,7 +473,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -481,7 +481,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -489,7 +489,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>260726</v>
+        <v>261005</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -505,7 +505,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -521,7 +521,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>2040</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="14" x14ac:dyDescent="0.3">

</xml_diff>